<commit_message>
Açık tema ve PDF tabanlı arama sistemi aktif edildi
</commit_message>
<xml_diff>
--- a/COMOROS_SIRKULER/Sirkuler_PDFleri/GBI_Sirkuler_Analizi_Turkce.xlsx
+++ b/COMOROS_SIRKULER/Sirkuler_PDFleri/GBI_Sirkuler_Analizi_Turkce.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>GBI Sirküler Dosyası</t>
+          <t>GBI Sirkuler Dosyası</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -466,27 +466,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Circular 01165_2018.07.16_validity of color copies of original documents on-board vessels flying under Comoros flag</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Genelge 01165_2018.07.16_Komor bayrağı taşıyan gemilerdeki orijinal belgelerin renkli kopyalarının geçerliliği</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular 01165_2018.07.16_validity of color copies of original documents on-board vessels flying under Comoros flag on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Genelge 01165_2018.07.16_Komor bayrağı taşıyan gemilerdeki orijinal belgelerin renkli kopyalarının geçerliliği ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -503,27 +503,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Approved_P&amp;I_list</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Approved_P&amp;I_list</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Approved_P&amp;I_list on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Approved_P&amp;I_list ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -535,32 +535,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>Klas / RO Yetkileri</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Authorized Recognized Organizations</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Yetkili Tanınan Kuruluşlar</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Authorized Recognized Organizations on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Yetkili Tanınan Kuruluşlar ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -577,27 +577,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Circular-Procedures related to the certification of vessels according to Maritime Labor Convention 2006</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Denizcilik Çalışma Sözleşmesi 2006'ya göre gemilerin sertifikalandırılmasına ilişkin Genelge-Prosedürler</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular-Procedures related to the certification of vessels according to Maritime Labor Convention 2006 on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Denizcilik Çalışma Sözleşmesi 2006'ya göre gemilerin sertifikalandırılmasına ilişkin Genelge-Prosedürler ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -609,32 +609,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>Statüter / Donanım</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Procedures on the Issuance of an Exemption Certificate</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Muafiyet Belgesi Verilme İşlemleri</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Procedures on the Issuance of an Exemption Certificate on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Muafiyet Belgesi Verilme İşlemleri ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -651,27 +651,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Nairobi International Convention on the Removal_of Wrecks, 2007</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Enkazların Kaldırılmasına İlişkin Nairobi Uluslararası Sözleşmesi, 2007</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Nairobi Convention 2007</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Nairobi International Convention on the Removal_of Wrecks, 2007 on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Enkazların Kaldırılmasına İlişkin Nairobi Uluslararası Sözleşmesi, 2007 ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -688,27 +688,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Circular 21 NOVEL CORONAVIRUS GUIDANCE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Genelge 21 YENİ KORONAVİRÜS REHBERİ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular 21 NOVEL CORONAVIRUS GUIDANCE on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Genelge 21 YENİ KORONAVİRÜS REHBERİ ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -725,27 +725,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Principles of Safe Manning</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Güvenli Personel Taşıma İlkeleri</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Principles of Safe Manning on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Güvenli Personel Taşıma İlkeleri ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -762,27 +762,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>International Convention On Civil Liability For-Oil Pollution Damage, 1992</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Petrol Kirliliğinden Kaynaklanan Zararlara İlişkin Hukuki Sorumluluk Uluslararası Sözleşmesi, 1992</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>CLC 1992 / Bunkers Convention</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning International Convention On Civil Liability For-Oil Pollution Damage, 1992 on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Petrol Kirliliğinden Kaynaklanan Zararlara İlişkin Hukuki Sorumluluk Uluslararası Sözleşmesi, 1992 ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -799,27 +799,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Circular 24 CORONAVIRUS (COVID-19)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Genelge 24 KORONAVİRÜS (COVID-19)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular 24 CORONAVIRUS (COVID-19) on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Genelge 24 KORONAVİRÜS (COVID-19) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -836,27 +836,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Circular – Renewal of Flag Certificates</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Genelge – Bayrak Sertifikalarının Yenilenmesi</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular – Renewal of Flag Certificates on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Genelge – Bayrak Sertifikalarının Yenilenmesi ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -868,32 +868,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>ISSC / ISPS</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Use of Privately Contracted Armed Security_Personnel (PCASP) on Board</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Gemide Özel Sözleşmeli Silahlı Güvenlik Personelinin (PCASP) Kullanımı</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ISPS Code</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Use of Privately Contracted Armed Security_Personnel (PCASP) on Board on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gemide Özel Sözleşmeli Silahlı Güvenlik Personelinin (PCASP) Kullanımı ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -910,27 +910,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>CONTINUOUS SYNOPSIS RECORD (CSR)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>SÜREKLİ ÖZET KAYDI (CSR)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning CONTINUOUS SYNOPSIS RECORD (CSR) on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde SÜREKLİ ÖZET KAYDI (CSR) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -942,32 +942,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>Statüter / Donanım</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>International Convention of Civil Liability for Bunker Oil Pollution Damage of 2001 (Bunkers Convention)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>2001 tarihli Bunker Petrol Kirliliği Zararına İlişkin Hukuki Sorumluluk Uluslararası Sözleşmesi (Bunkerler Sözleşmesi)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>CLC 1992 / Bunkers Convention</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning International Convention of Civil Liability for Bunker Oil Pollution Damage of 2001 (Bunkers Convention) on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde 2001 tarihli Bunker Petrol Kirliliği Zararına İlişkin Hukuki Sorumluluk Uluslararası Sözleşmesi (Bunkerler Sözleşmesi) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -979,32 +979,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>Statüter / Donanım</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Circular Coronavirus (COVID 19) – WHO Guidance to Promote Public Health Measures on Cargo Ships and Fishing Vessels</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Dairesel Coronavirüs (COVID 19) – Kargo Gemileri ve Balıkçı Gemilerinde Halk Sağlığı Önlemlerinin Geliştirilmesine İlişkin DSÖ Rehberi</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular Coronavirus (COVID 19) – WHO Guidance to Promote Public Health Measures on Cargo Ships and Fishing Vessels on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Dairesel Coronavirüs (COVID 19) – Kargo Gemileri ve Balıkçı Gemilerinde Halk Sağlığı Önlemlerinin Geliştirilmesine İlişkin DSÖ Rehberi ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -1021,27 +1021,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Circular INVENTORY OF HAZARDOUS MATERIALS (IHM) FOR SHIPS_CALLING AT EU PORTS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>AB LİMANLARINDA GEMİLER İÇİN TEHLİKELİ MADDELER (IHM) Genelgesi Envanteri</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular INVENTORY OF HAZARDOUS MATERIALS (IHM) FOR SHIPS_CALLING AT EU PORTS on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde AB LİMANLARINDA GEMİLER İÇİN TEHLİKELİ MADDELER (IHM) Genelgesi Envanteri ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -1053,32 +1053,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>Statüter / Donanım</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Collection And Reporting Requirements For The Ship Fuel Oil Consumption Data</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Gemi Akaryakıt Tüketim Verilerinin Toplanması ve Raporlanması Gereksinimleri</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Collection And Reporting Requirements For The Ship Fuel Oil Consumption Data on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gemi Akaryakıt Tüketim Verilerinin Toplanması ve Raporlanması Gereksinimleri ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -1095,27 +1095,27 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Circular Policy of Detentions</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Gözaltılara İlişkin Genelge Politikası</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular Policy of Detentions on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gözaltılara İlişkin Genelge Politikası ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -1132,27 +1132,27 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Obligations of Owners/Managers/Operators Related to the Safe and Secure Operation of Ships</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Gemi Sahiplerinin/Yöneticilerinin/İşletmecilerinin Gemilerin Emniyetli ve Emniyetli Operasyonuna İlişkin Yükümlülükleri</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Obligations of Owners/Managers/Operators Related to the Safe and Secure Operation of Ships on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gemi Sahiplerinin/Yöneticilerinin/İşletmecilerinin Gemilerin Emniyetli ve Emniyetli Operasyonuna İlişkin Yükümlülükleri ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -1169,27 +1169,27 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Issuance of Flag Endorsements According to STCW, as amended requirements</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Değiştirilen gereksinimler doğrultusunda STCW'ye göre Bayrak Onaylarının Verilmesi</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>STCW 78/95</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Issuance of Flag Endorsements According to STCW, as amended requirements on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Değiştirilen gereksinimler doğrultusunda STCW'ye göre Bayrak Onaylarının Verilmesi ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -1206,27 +1206,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>AUTHORIZATION-FOR-SERVICE-PROVIDERS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>HİZMET SAĞLAYICILAR İÇİN YETKİLENDİRME</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning AUTHORIZATION-FOR-SERVICE-PROVIDERS on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde HİZMET SAĞLAYICILAR İÇİN YETKİLENDİRME ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -1238,32 +1238,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>MLC</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Circular 36 Issuance of Seafarer’s Identification and Record Book (SIRB)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Genelge 36 Gemiadamı Kimlik ve Kayıt Defterinin Düzenlenmesi (SIRB)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular 36 Issuance of Seafarer’s Identification and Record Book (SIRB) on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Genelge 36 Gemiadamı Kimlik ve Kayıt Defterinin Düzenlenmesi (SIRB) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
@@ -1275,39 +1275,39 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>Statüter / Donanım</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Circular Authorization for Service Providers_LSA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Hizmet Sağlayıcılar için Genel Yetkilendirme_LSA</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular Authorization for Service Providers_LSA on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Hizmet Sağlayıcılar için Genel Yetkilendirme_LSA ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Circular-Coronavirus-COVID-19-%E2%80%93-Guidance-Relating-to-the-Postponement-Extension-of-Statutory-Certification-Services-2Updated.pdf</t>
+          <t>Circular-Resting-Hours-IMO-Guidelines-on-Fatigue.pdf</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1317,145 +1317,145 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Circular Resting Hours &amp; IMO Guidelines on Fatigue</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Döngüsel Dinlenme Saatleri ve Yorgunluğa İlişkin IMO Kılavuzları</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular Resting Hours &amp; IMO Guidelines on Fatigue on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Döngüsel Dinlenme Saatleri ve Yorgunluğa İlişkin IMO Kılavuzları ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Circular-Resting-Hours-IMO-Guidelines-on-Fatigue.pdf</t>
+          <t>Circular-Ship-Security-Level-III-within-the-Eastern-Mediterranean-Sea-Area.pdf</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>ISSC / ISPS</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Circular Ship Security Level III within the Eastern Mediterranean Sea Area</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Doğu Akdeniz Bölgesinde Dairesel Gemi Güvenlik Seviyesi III</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ISPS Code</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular Ship Security Level III within the Eastern Mediterranean Sea Area on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Doğu Akdeniz Bölgesinde Dairesel Gemi Güvenlik Seviyesi III ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Circular-Ship-Security-Level-III-within-the-Eastern-Mediterranean-Sea-Area.pdf</t>
+          <t>COVID-19 - Guidance Relating to the Certification of Seafarers.pdf</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>MLC</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>COVID-19 – Guidance Relating to the Certification of Seafarers</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>COVID-19 – Denizcilerin Sertifikalandırılmasına İlişkin Rehber</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning COVID-19 – Guidance Relating to the Certification of Seafarers on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde COVID-19 – Denizcilerin Sertifikalandırılmasına İlişkin Rehber ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>COVID-19 - Guidance Relating to the Certification of Seafarers.pdf</t>
+          <t>Crew Dispensation Letter_20_01857_com.pdf</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MLC</t>
+          <t>MLC, Statüter / Donanım</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Coronavirus (COVID-19) – Guidance relating to the certification of</t>
+          <t>Crew Dispensation Letter_20_01857</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Coronavirüs (COVID-19) – Sertifikasyona ilişkin kılavuz</t>
+          <t>Mürettebat Muafiyet Mektubu_20_01857</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Crew Dispensation Letter_20_01857 on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Mürettebat Muafiyet Mektubu_20_01857 ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Crew Dispensation Letter_20_01857_com.pdf</t>
+          <t>GUIDANCE-TO-POSTPONEMENT-OF-SURVEYS-AND-SEVICES-20210104_21_01855_com_rev_3.pdf</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1465,34 +1465,34 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>GUIDANCE-TO-POSTPONEMENT-OF-SURVEYS-AND-SERVICES-20210104_21_01855_com_rev_3</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANKETLERİN-VE-HİZMETLERİN-ERTELENMESİ İÇİN REHBERLİK-20210104_21_01855_com_rev_3</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning GUIDANCE-TO-POSTPONEMENT-OF-SURVEYS-AND-SERVICES-20210104_21_01855_com_rev_3 on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde ANKETLERİN-VE-HİZMETLERİN-ERTELENMESİ İÇİN REHBERLİK-20210104_21_01855_com_rev_3 ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>GUIDANCE-TO-POSTPONEMENT-OF-SURVEYS-AND-SEVICES-20210104_21_01855_com_rev_3.pdf</t>
+          <t>Insurance Companies Accepted by ANAM.pdf</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1502,71 +1502,71 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Insurance Companies Accepted by ANAM</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM'ın Kabul Ettiği Sigorta Şirketleri</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Insurance Companies Accepted by ANAM on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde ANAM'ın Kabul Ettiği Sigorta Şirketleri ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Insurance Companies Accepted by ANAM.pdf</t>
+          <t>List of Approved Radio Accounting Authorities by ANAM.pdf</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>Statüter / Donanım</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>List of Approved Radio Accounting Authorities</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Onaylanmış Radyo Muhasebe Yetkililerinin Listesi</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning List of Approved Radio Accounting Authorities on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Onaylanmış Radyo Muhasebe Yetkililerinin Listesi ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>List of Approved Radio Accounting Authorities by ANAM.pdf</t>
+          <t>Long-Range Identification and Tracking (LRIT) of Ships.pdf</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1576,108 +1576,108 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Long-Range Identification and Tracking (LRIT) of Ships</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Gemilerin Uzun Menzilli Tanımlanması ve Takibi (LRIT)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Long-Range Identification and Tracking (LRIT) of Ships on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gemilerin Uzun Menzilli Tanımlanması ve Takibi (LRIT) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Long-Range Identification and Tracking (LRIT) of Ships.pdf</t>
+          <t>Policy on Ballast Water Management Convention 2004.pdf</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>Statüter / Donanım</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Policy on Ballast Water Management Convention 2004</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Balast Suyu Yönetimi Politikası Sözleşmesi 2004</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Policy on Ballast Water Management Convention 2004 on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Balast Suyu Yönetimi Politikası Sözleşmesi 2004 ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Policy on Ballast Water Management Convention 2004.pdf</t>
+          <t>Reefer Vessel Prohibited to Trade with Fishing Activities.pdf</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Statüter / Donanım, Klas / RO Yetkileri</t>
+          <t>Genel / Diğer</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Reefer Vessel Prohibited to Trade with Fishing Activities</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Soğutmalı Geminin Balıkçılık Faaliyetleriyle Ticaret Yapması Yasaktır</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>1.1. The purpose of this Circular is to inform all parties concerned about the procedures which shall be followed when a vessel which flies the flag of Comoros is surveyed according to the requirements of “Ballast Water Management Convention 2004”. 1.2. The Convention will enter into force on 08 September 2017 and all vessels flying the flag of Comoros shall comply with its requirements....</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Reefer Vessel Prohibited to Trade with Fishing Activities on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>1.1. Bu Genelgenin amacı, Komor bayrağı taşıyan bir geminin “Balast Suyu Yönetimi Sözleşmesi 2004” gerekliliklerine göre sörvey edilmesi durumunda izlenecek prosedürler konusunda ilgili tüm tarafları bilgilendirmektir. 1.2. Sözleşme 08 Eylül 2017 tarihinde yürürlüğe girecek ve Komor bayrağını taşıyan tüm gemiler bu sözleşmenin gerekliliklerine uyacaktır....</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Soğutmalı Geminin Balıkçılık Faaliyetleriyle Ticaret Yapması Yasaktır ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Reefer Vessel Prohibited to Trade with Fishing Activities.pdf</t>
+          <t>Reporting of Issued Certificates.pdf</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1687,34 +1687,34 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Reporting of Issued Certificates</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Verilen Sertifikaların Raporlanması</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Reporting of Issued Certificates on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Verilen Sertifikaların Raporlanması ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Reporting of Issued Certificates.pdf</t>
+          <t>Reporting of PSC Inspections_Detentions and Incidents.pdf</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1724,71 +1724,71 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Reporting of PSC Inspections/Detentions and Incidents</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>PSC Denetimleri/Gözaltılar ve Olayların Raporlanması</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Reporting of PSC Inspections/Detentions and Incidents on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde PSC Denetimleri/Gözaltılar ve Olayların Raporlanması ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Reporting of PSC Inspections_Detentions and Incidents.pdf</t>
+          <t>SHIP SECURITY ALERT SYSTEM (SSAS)-2019.pdf</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>ISSC / ISPS</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Ship Security Alert System (SSAS)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Gemi Güvenlik Uyarı Sistemi (SSAS)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ISPS Code</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Ship Security Alert System (SSAS) on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gemi Güvenlik Uyarı Sistemi (SSAS) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SHIP SECURITY ALERT SYSTEM (SSAS)-2019.pdf</t>
+          <t>Trading in Prohibited Area.pdf</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1798,34 +1798,34 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Trading in Prohibited Area</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Yasak Bölgede Ticaret</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Trading in Prohibited Area on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Yasak Bölgede Ticaret ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Trading in Prohibited Area.pdf</t>
+          <t>Type Approvals and Criteria to the Satisfaction of the Administration.pdf</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1835,34 +1835,34 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Type Approvals and Criteria to the Satisfaction of the Administration</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Tip Onayları ve İdarenin Memnuniyetine İlişkin Kriterler</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Type Approvals and Criteria to the Satisfaction of the Administration on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Tip Onayları ve İdarenin Memnuniyetine İlişkin Kriterler ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Type Approvals and Criteria to the Satisfaction of the Administration.pdf</t>
+          <t>Circular-Coronavirus-COVID-19-%E2%80%93-Guidance-Relating-to-the-Postponement-Extension-of-Statutory-Certification-Services-2Updated.pdf</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1872,27 +1872,27 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Circular Coronavirus Covid 19 %E2%80%93 Guidance Relating To The Postponement Extension Of Statutory Certification Services 2Updated</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Genelge Coronavirüs Covid 19 %E2%80%93 Yasal Sertifikasyon Hizmetlerinin Ertelenmesinin Uzatılmasına İlişkin Rehberlik 2Güncellendi</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>This official circular provides guidance and regulatory criteria concerning Circular Coronavirus Covid 19 %E2%80%93 Guidance Relating To The Postponement Extension Of Statutory Certification Services 2Updated.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Bu resmi genelge, Genelge Coronavirüs Covid 19 %E2%80%93 Yasal Sertifikasyon Hizmetlerinin Ertelenmesinin Uzatılmasına İlişkin Rehberlik 2Güncellendi ile ilgili rehberlik ve düzenleyici kriterler sağlamaktadır.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Unifed database schema, added recommendations column, fixed selectbox bugs and Spanish vertical layout parsing
</commit_message>
<xml_diff>
--- a/COMOROS_SIRKULER/Sirkuler_PDFleri/GBI_Sirkuler_Analizi_Turkce.xlsx
+++ b/COMOROS_SIRKULER/Sirkuler_PDFleri/GBI_Sirkuler_Analizi_Turkce.xlsx
@@ -413,43 +413,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>GBI Sirkuler Dosyası</t>
+          <t>Filename</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>İlgili Sertifika Kategorisi</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Konu (İngilizce)</t>
+          <t>Subject_EN</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Konu (TÜRKÇE)</t>
+          <t>Subject_TR</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Kural Dayanağı / Referanslar</t>
+          <t>References</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Özet Açıklama (İngilizce)</t>
+          <t>Summary_EN</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Özet Açıklama (TÜRKÇE)</t>
+          <t>Summary_TR</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Recommendations_TR</t>
         </is>
       </c>
     </row>
@@ -489,6 +494,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Genelge 01165_2018.07.16_Komor bayrağı taşıyan gemilerdeki orijinal belgelerin renkli kopyalarının geçerliliği ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -526,6 +536,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Approved_P&amp;I_list ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -563,6 +578,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Yetkili Tanınan Kuruluşlar ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1. RO (Sınıf Kuruluşu) yetkilendirme limitlerini ve sörveyör kılavuz maddelerini kontrol edin. 2. Sörvey sırasında yetkili RO formlarının kullanıldığını teyit edin.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -600,6 +620,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Denizcilik Çalışma Sözleşmesi 2006'ya göre gemilerin sertifikalandırılmasına ilişkin Genelge-Prosedürler ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -637,6 +662,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Muafiyet Belgesi Verilme İşlemleri ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1. LSA (Can kurtarma araçları) ve FFA (Yangınla mücadele) ekipmanlarının bakım ve servis kayıtlarını kontrol edin. 2. Balast suyu yönetim planı ve kayıt defterinin en güncel IMO kurallarına göre tutulduğunu doğrulayın. 3. İdarenin (Flag Administration) yazılı resmi izni olmadan hiçbir SOLAS/MARPOL muafiyeti (exemption) uygulamayın.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -674,6 +704,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Enkazların Kaldırılmasına İlişkin Nairobi Uluslararası Sözleşmesi, 2007 ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -711,6 +746,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Genelge 21 YENİ KORONAVİRÜS REHBERİ ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -748,6 +788,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Güvenli Personel Taşıma İlkeleri ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -785,6 +830,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Petrol Kirliliğinden Kaynaklanan Zararlara İlişkin Hukuki Sorumluluk Uluslararası Sözleşmesi, 1992 ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -822,6 +872,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Genelge 24 KORONAVİRÜS (COVID-19) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -859,6 +914,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Genelge – Bayrak Sertifikalarının Yenilenmesi ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -896,6 +956,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gemide Özel Sözleşmeli Silahlı Güvenlik Personelinin (PCASP) Kullanımı ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1. Gemi Güvenlik Planını (SSP) ve güvenlik seviyesi talimatlarını güncelleyin. 2. SSAS (Gemi Güvenlik Uyarı Sistemi) alıcı ayarlarını ve test prosedürlerini kontrol edin. 3. Şirket Güvenlik Sorumlusu (CSO) iletişim bilgilerinin gemide asılı olduğunu teyit edin.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -933,6 +998,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde SÜREKLİ ÖZET KAYDI (CSR) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -970,6 +1040,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde 2001 tarihli Bunker Petrol Kirliliği Zararına İlişkin Hukuki Sorumluluk Uluslararası Sözleşmesi (Bunkerler Sözleşmesi) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1. LSA (Can kurtarma araçları) ve FFA (Yangınla mücadele) ekipmanlarının bakım ve servis kayıtlarını kontrol edin. 2. Balast suyu yönetim planı ve kayıt defterinin en güncel IMO kurallarına göre tutulduğunu doğrulayın. 3. İdarenin (Flag Administration) yazılı resmi izni olmadan hiçbir SOLAS/MARPOL muafiyeti (exemption) uygulamayın.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1007,6 +1082,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Dairesel Coronavirüs (COVID 19) – Kargo Gemileri ve Balıkçı Gemilerinde Halk Sağlığı Önlemlerinin Geliştirilmesine İlişkin DSÖ Rehberi ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1. LSA (Can kurtarma araçları) ve FFA (Yangınla mücadele) ekipmanlarının bakım ve servis kayıtlarını kontrol edin. 2. Balast suyu yönetim planı ve kayıt defterinin en güncel IMO kurallarına göre tutulduğunu doğrulayın. 3. İdarenin (Flag Administration) yazılı resmi izni olmadan hiçbir SOLAS/MARPOL muafiyeti (exemption) uygulamayın.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1044,6 +1124,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde AB LİMANLARINDA GEMİLER İÇİN TEHLİKELİ MADDELER (IHM) Genelgesi Envanteri ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1081,6 +1166,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gemi Akaryakıt Tüketim Verilerinin Toplanması ve Raporlanması Gereksinimleri ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1. LSA (Can kurtarma araçları) ve FFA (Yangınla mücadele) ekipmanlarının bakım ve servis kayıtlarını kontrol edin. 2. Balast suyu yönetim planı ve kayıt defterinin en güncel IMO kurallarına göre tutulduğunu doğrulayın. 3. İdarenin (Flag Administration) yazılı resmi izni olmadan hiçbir SOLAS/MARPOL muafiyeti (exemption) uygulamayın.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1118,6 +1208,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gözaltılara İlişkin Genelge Politikası ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1155,6 +1250,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gemi Sahiplerinin/Yöneticilerinin/İşletmecilerinin Gemilerin Emniyetli ve Emniyetli Operasyonuna İlişkin Yükümlülükleri ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1192,6 +1292,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Değiştirilen gereksinimler doğrultusunda STCW'ye göre Bayrak Onaylarının Verilmesi ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1229,6 +1334,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde HİZMET SAĞLAYICILAR İÇİN YETKİLENDİRME ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1266,6 +1376,11 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Genelge 36 Gemiadamı Kimlik ve Kayıt Defterinin Düzenlenmesi (SIRB) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>1. MLC 2006 mali güvence sigorta sertifikalarının güncel basılı kopyalarını gemide herkesin görebileceği bir yere asın. 2. Gemiadamı iş sözleşmelerinin (SEA) asgari ücret, izin ve bayrak kanunu kurallarına uygunluğunu teyit edin. 3. Çalışma ve dinlenme saatleri kayıtlarının (Rest Hours) eksiksiz tutulduğunu kontrol edin.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1303,11 +1418,16 @@
           <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Hizmet Sağlayıcılar için Genel Yetkilendirme_LSA ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>1. LSA (Can kurtarma araçları) ve FFA (Yangınla mücadele) ekipmanlarının bakım ve servis kayıtlarını kontrol edin. 2. Balast suyu yönetim planı ve kayıt defterinin en güncel IMO kurallarına göre tutulduğunu doğrulayın. 3. İdarenin (Flag Administration) yazılı resmi izni olmadan hiçbir SOLAS/MARPOL muafiyeti (exemption) uygulamayın.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Circular-Resting-Hours-IMO-Guidelines-on-Fatigue.pdf</t>
+          <t>Circular-Coronavirus-COVID-19-%E2%80%93-Guidance-Relating-to-the-Postponement-Extension-of-Statutory-Certification-Services-2Updated.pdf</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1317,12 +1437,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Circular Resting Hours &amp; IMO Guidelines on Fatigue</t>
+          <t>Circular Coronavirus Covid 19 %E2%80%93 Guidance Relating To The Postponement Extension Of Statutory Certification Services 2Updated</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Döngüsel Dinlenme Saatleri ve Yorgunluğa İlişkin IMO Kılavuzları</t>
+          <t>Genelge Coronavirüs Covid 19 %E2%80%93 Yasal Sertifikasyon Hizmetlerinin Ertelenmesinin Uzatılmasına İlişkin Rehberlik 2Güncellendi</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1332,108 +1452,123 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular Resting Hours &amp; IMO Guidelines on Fatigue on Comoros flagged vessels.</t>
+          <t>This official circular provides guidance and regulatory criteria concerning Circular Coronavirus Covid 19 %E2%80%93 Guidance Relating To The Postponement Extension Of Statutory Certification Services 2Updated.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Döngüsel Dinlenme Saatleri ve Yorgunluğa İlişkin IMO Kılavuzları ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi genelge, Genelge Coronavirüs Covid 19 %E2%80%93 Yasal Sertifikasyon Hizmetlerinin Ertelenmesinin Uzatılmasına İlişkin Rehberlik 2Güncellendi ile ilgili rehberlik ve düzenleyici kriterler sağlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Circular-Ship-Security-Level-III-within-the-Eastern-Mediterranean-Sea-Area.pdf</t>
+          <t>Circular-Resting-Hours-IMO-Guidelines-on-Fatigue.pdf</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ISSC / ISPS</t>
+          <t>Genel / Diğer</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Circular Ship Security Level III within the Eastern Mediterranean Sea Area</t>
+          <t>Circular Resting Hours &amp; IMO Guidelines on Fatigue</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Doğu Akdeniz Bölgesinde Dairesel Gemi Güvenlik Seviyesi III</t>
+          <t>Döngüsel Dinlenme Saatleri ve Yorgunluğa İlişkin IMO Kılavuzları</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ISPS Code</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular Ship Security Level III within the Eastern Mediterranean Sea Area on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular Resting Hours &amp; IMO Guidelines on Fatigue on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Doğu Akdeniz Bölgesinde Dairesel Gemi Güvenlik Seviyesi III ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Döngüsel Dinlenme Saatleri ve Yorgunluğa İlişkin IMO Kılavuzları ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>COVID-19 - Guidance Relating to the Certification of Seafarers.pdf</t>
+          <t>Circular-Ship-Security-Level-III-within-the-Eastern-Mediterranean-Sea-Area.pdf</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MLC</t>
+          <t>ISSC / ISPS</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>COVID-19 – Guidance Relating to the Certification of Seafarers</t>
+          <t>Circular Ship Security Level III within the Eastern Mediterranean Sea Area</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>COVID-19 – Denizcilerin Sertifikalandırılmasına İlişkin Rehber</t>
+          <t>Doğu Akdeniz Bölgesinde Dairesel Gemi Güvenlik Seviyesi III</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ANAM Circular / Yönerge</t>
+          <t>ISPS Code</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning COVID-19 – Guidance Relating to the Certification of Seafarers on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Circular Ship Security Level III within the Eastern Mediterranean Sea Area on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde COVID-19 – Denizcilerin Sertifikalandırılmasına İlişkin Rehber ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Doğu Akdeniz Bölgesinde Dairesel Gemi Güvenlik Seviyesi III ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>1. Gemi Güvenlik Planını (SSP) ve güvenlik seviyesi talimatlarını güncelleyin. 2. SSAS (Gemi Güvenlik Uyarı Sistemi) alıcı ayarlarını ve test prosedürlerini kontrol edin. 3. Şirket Güvenlik Sorumlusu (CSO) iletişim bilgilerinin gemide asılı olduğunu teyit edin.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Crew Dispensation Letter_20_01857_com.pdf</t>
+          <t>COVID-19 - Guidance Relating to the Certification of Seafarers.pdf</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MLC, Statüter / Donanım</t>
+          <t>MLC</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Crew Dispensation Letter_20_01857</t>
+          <t>COVID-19 – Guidance Relating to the Certification of Seafarers</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Mürettebat Muafiyet Mektubu_20_01857</t>
+          <t>COVID-19 – Denizcilerin Sertifikalandırılmasına İlişkin Rehber</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1443,34 +1578,39 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning Crew Dispensation Letter_20_01857 on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning COVID-19 – Guidance Relating to the Certification of Seafarers on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Mürettebat Muafiyet Mektubu_20_01857 ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde COVID-19 – Denizcilerin Sertifikalandırılmasına İlişkin Rehber ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>1. MLC 2006 mali güvence sigorta sertifikalarının güncel basılı kopyalarını gemide herkesin görebileceği bir yere asın. 2. Gemiadamı iş sözleşmelerinin (SEA) asgari ücret, izin ve bayrak kanunu kurallarına uygunluğunu teyit edin. 3. Çalışma ve dinlenme saatleri kayıtlarının (Rest Hours) eksiksiz tutulduğunu kontrol edin.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GUIDANCE-TO-POSTPONEMENT-OF-SURVEYS-AND-SEVICES-20210104_21_01855_com_rev_3.pdf</t>
+          <t>Crew Dispensation Letter_20_01857_com.pdf</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>MLC, Statüter / Donanım</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>GUIDANCE-TO-POSTPONEMENT-OF-SURVEYS-AND-SERVICES-20210104_21_01855_com_rev_3</t>
+          <t>Crew Dispensation Letter_20_01857</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ANKETLERİN-VE-HİZMETLERİN-ERTELENMESİ İÇİN REHBERLİK-20210104_21_01855_com_rev_3</t>
+          <t>Mürettebat Muafiyet Mektubu_20_01857</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1480,19 +1620,24 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning GUIDANCE-TO-POSTPONEMENT-OF-SURVEYS-AND-SERVICES-20210104_21_01855_com_rev_3 on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Crew Dispensation Letter_20_01857 on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde ANKETLERİN-VE-HİZMETLERİN-ERTELENMESİ İÇİN REHBERLİK-20210104_21_01855_com_rev_3 ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Mürettebat Muafiyet Mektubu_20_01857 ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>1. MLC 2006 mali güvence sigorta sertifikalarının güncel basılı kopyalarını gemide herkesin görebileceği bir yere asın. 2. Gemiadamı iş sözleşmelerinin (SEA) asgari ücret, izin ve bayrak kanunu kurallarına uygunluğunu teyit edin. 3. Çalışma ve dinlenme saatleri kayıtlarının (Rest Hours) eksiksiz tutulduğunu kontrol edin.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Insurance Companies Accepted by ANAM.pdf</t>
+          <t>GUIDANCE-TO-POSTPONEMENT-OF-SURVEYS-AND-SEVICES-20210104_21_01855_com_rev_3.pdf</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1502,12 +1647,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Insurance Companies Accepted by ANAM</t>
+          <t>GUIDANCE-TO-POSTPONEMENT-OF-SURVEYS-AND-SERVICES-20210104_21_01855_com_rev_3</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>ANAM'ın Kabul Ettiği Sigorta Şirketleri</t>
+          <t>ANKETLERİN-VE-HİZMETLERİN-ERTELENMESİ İÇİN REHBERLİK-20210104_21_01855_com_rev_3</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1517,34 +1662,39 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning Insurance Companies Accepted by ANAM on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning GUIDANCE-TO-POSTPONEMENT-OF-SURVEYS-AND-SERVICES-20210104_21_01855_com_rev_3 on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde ANAM'ın Kabul Ettiği Sigorta Şirketleri ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde ANKETLERİN-VE-HİZMETLERİN-ERTELENMESİ İÇİN REHBERLİK-20210104_21_01855_com_rev_3 ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>List of Approved Radio Accounting Authorities by ANAM.pdf</t>
+          <t>Insurance Companies Accepted by ANAM.pdf</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Statüter / Donanım</t>
+          <t>Genel / Diğer</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>List of Approved Radio Accounting Authorities</t>
+          <t>Insurance Companies Accepted by ANAM</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Onaylanmış Radyo Muhasebe Yetkililerinin Listesi</t>
+          <t>ANAM'ın Kabul Ettiği Sigorta Şirketleri</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1554,34 +1704,39 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning List of Approved Radio Accounting Authorities on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Insurance Companies Accepted by ANAM on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Onaylanmış Radyo Muhasebe Yetkililerinin Listesi ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde ANAM'ın Kabul Ettiği Sigorta Şirketleri ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Long-Range Identification and Tracking (LRIT) of Ships.pdf</t>
+          <t>List of Approved Radio Accounting Authorities by ANAM.pdf</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>Statüter / Donanım</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Long-Range Identification and Tracking (LRIT) of Ships</t>
+          <t>List of Approved Radio Accounting Authorities</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Gemilerin Uzun Menzilli Tanımlanması ve Takibi (LRIT)</t>
+          <t>Onaylanmış Radyo Muhasebe Yetkililerinin Listesi</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1591,34 +1746,39 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning Long-Range Identification and Tracking (LRIT) of Ships on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning List of Approved Radio Accounting Authorities on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gemilerin Uzun Menzilli Tanımlanması ve Takibi (LRIT) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Onaylanmış Radyo Muhasebe Yetkililerinin Listesi ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>1. LSA (Can kurtarma araçları) ve FFA (Yangınla mücadele) ekipmanlarının bakım ve servis kayıtlarını kontrol edin. 2. Balast suyu yönetim planı ve kayıt defterinin en güncel IMO kurallarına göre tutulduğunu doğrulayın. 3. İdarenin (Flag Administration) yazılı resmi izni olmadan hiçbir SOLAS/MARPOL muafiyeti (exemption) uygulamayın.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Policy on Ballast Water Management Convention 2004.pdf</t>
+          <t>Long-Range Identification and Tracking (LRIT) of Ships.pdf</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Statüter / Donanım</t>
+          <t>Genel / Diğer</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Policy on Ballast Water Management Convention 2004</t>
+          <t>Long-Range Identification and Tracking (LRIT) of Ships</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Balast Suyu Yönetimi Politikası Sözleşmesi 2004</t>
+          <t>Gemilerin Uzun Menzilli Tanımlanması ve Takibi (LRIT)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1628,34 +1788,39 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning Policy on Ballast Water Management Convention 2004 on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Long-Range Identification and Tracking (LRIT) of Ships on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Balast Suyu Yönetimi Politikası Sözleşmesi 2004 ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gemilerin Uzun Menzilli Tanımlanması ve Takibi (LRIT) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>1. LRIT uygunluk test raporunu (CTR) gemide orijinal olarak bulundurun ve veri iletiminin kesintisiz sağlandığını test edin.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Reefer Vessel Prohibited to Trade with Fishing Activities.pdf</t>
+          <t>Policy on Ballast Water Management Convention 2004.pdf</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>Statüter / Donanım</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Reefer Vessel Prohibited to Trade with Fishing Activities</t>
+          <t>Policy on Ballast Water Management Convention 2004</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Soğutmalı Geminin Balıkçılık Faaliyetleriyle Ticaret Yapması Yasaktır</t>
+          <t>Balast Suyu Yönetimi Politikası Sözleşmesi 2004</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1665,19 +1830,24 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning Reefer Vessel Prohibited to Trade with Fishing Activities on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Policy on Ballast Water Management Convention 2004 on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Soğutmalı Geminin Balıkçılık Faaliyetleriyle Ticaret Yapması Yasaktır ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Balast Suyu Yönetimi Politikası Sözleşmesi 2004 ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>1. LSA (Can kurtarma araçları) ve FFA (Yangınla mücadele) ekipmanlarının bakım ve servis kayıtlarını kontrol edin. 2. Balast suyu yönetim planı ve kayıt defterinin en güncel IMO kurallarına göre tutulduğunu doğrulayın. 3. İdarenin (Flag Administration) yazılı resmi izni olmadan hiçbir SOLAS/MARPOL muafiyeti (exemption) uygulamayın.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Reporting of Issued Certificates.pdf</t>
+          <t>Reefer Vessel Prohibited to Trade with Fishing Activities.pdf</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1687,12 +1857,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Reporting of Issued Certificates</t>
+          <t>Reefer Vessel Prohibited to Trade with Fishing Activities</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Verilen Sertifikaların Raporlanması</t>
+          <t>Soğutmalı Geminin Balıkçılık Faaliyetleriyle Ticaret Yapması Yasaktır</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1702,19 +1872,24 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning Reporting of Issued Certificates on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Reefer Vessel Prohibited to Trade with Fishing Activities on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Verilen Sertifikaların Raporlanması ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Soğutmalı Geminin Balıkçılık Faaliyetleriyle Ticaret Yapması Yasaktır ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Reporting of PSC Inspections_Detentions and Incidents.pdf</t>
+          <t>Reporting of Issued Certificates.pdf</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1724,12 +1899,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Reporting of PSC Inspections/Detentions and Incidents</t>
+          <t>Reporting of Issued Certificates</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>PSC Denetimleri/Gözaltılar ve Olayların Raporlanması</t>
+          <t>Verilen Sertifikaların Raporlanması</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1739,93 +1914,108 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning Reporting of PSC Inspections/Detentions and Incidents on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Reporting of Issued Certificates on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde PSC Denetimleri/Gözaltılar ve Olayların Raporlanması ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Verilen Sertifikaların Raporlanması ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SHIP SECURITY ALERT SYSTEM (SSAS)-2019.pdf</t>
+          <t>Reporting of PSC Inspections_Detentions and Incidents.pdf</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ISSC / ISPS</t>
+          <t>Genel / Diğer</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Ship Security Alert System (SSAS)</t>
+          <t>Reporting of PSC Inspections/Detentions and Incidents</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Gemi Güvenlik Uyarı Sistemi (SSAS)</t>
+          <t>PSC Denetimleri/Gözaltılar ve Olayların Raporlanması</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ISPS Code</t>
+          <t>ANAM Circular / Yönerge</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning Ship Security Alert System (SSAS) on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Reporting of PSC Inspections/Detentions and Incidents on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gemi Güvenlik Uyarı Sistemi (SSAS) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde PSC Denetimleri/Gözaltılar ve Olayların Raporlanması ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>1. Yaklaşan sörvey/denetim tarih aralığını takip edin ve zamanında başvuru yapın. 2. PSC denetiminde eksiklik (code 17/30) alınması durumunda en geç 24 saat içinde bayrak idaresine ve RO'ya raporlayın.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Trading in Prohibited Area.pdf</t>
+          <t>SHIP SECURITY ALERT SYSTEM (SSAS)-2019.pdf</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Genel / Diğer</t>
+          <t>ISSC / ISPS</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Trading in Prohibited Area</t>
+          <t>Ship Security Alert System (SSAS)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Yasak Bölgede Ticaret</t>
+          <t>Gemi Güvenlik Uyarı Sistemi (SSAS)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ANAM Circular / Yönerge</t>
+          <t>ISPS Code</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning Trading in Prohibited Area on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Ship Security Alert System (SSAS) on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Yasak Bölgede Ticaret ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Gemi Güvenlik Uyarı Sistemi (SSAS) ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>1. Gemi Güvenlik Planını (SSP) ve güvenlik seviyesi talimatlarını güncelleyin. 2. SSAS (Gemi Güvenlik Uyarı Sistemi) alıcı ayarlarını ve test prosedürlerini kontrol edin. 3. Şirket Güvenlik Sorumlusu (CSO) iletişim bilgilerinin gemide asılı olduğunu teyit edin.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Type Approvals and Criteria to the Satisfaction of the Administration.pdf</t>
+          <t>Trading in Prohibited Area.pdf</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1835,12 +2025,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Type Approvals and Criteria to the Satisfaction of the Administration</t>
+          <t>Trading in Prohibited Area</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Tip Onayları ve İdarenin Memnuniyetine İlişkin Kriterler</t>
+          <t>Yasak Bölgede Ticaret</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1850,19 +2040,24 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>This official marine circular defines the guidelines and administrative procedures concerning Type Approvals and Criteria to the Satisfaction of the Administration on Comoros flagged vessels.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Trading in Prohibited Area on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Tip Onayları ve İdarenin Memnuniyetine İlişkin Kriterler ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Yasak Bölgede Ticaret ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Circular-Coronavirus-COVID-19-%E2%80%93-Guidance-Relating-to-the-Postponement-Extension-of-Statutory-Certification-Services-2Updated.pdf</t>
+          <t>Type Approvals and Criteria to the Satisfaction of the Administration.pdf</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1872,12 +2067,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Circular Coronavirus Covid 19 %E2%80%93 Guidance Relating To The Postponement Extension Of Statutory Certification Services 2Updated</t>
+          <t>Type Approvals and Criteria to the Satisfaction of the Administration</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Genelge Coronavirüs Covid 19 %E2%80%93 Yasal Sertifikasyon Hizmetlerinin Ertelenmesinin Uzatılmasına İlişkin Rehberlik 2Güncellendi</t>
+          <t>Tip Onayları ve İdarenin Memnuniyetine İlişkin Kriterler</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1887,12 +2082,17 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>This official circular provides guidance and regulatory criteria concerning Circular Coronavirus Covid 19 %E2%80%93 Guidance Relating To The Postponement Extension Of Statutory Certification Services 2Updated.</t>
+          <t>This official marine circular defines the guidelines and administrative procedures concerning Type Approvals and Criteria to the Satisfaction of the Administration on Comoros flagged vessels.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Bu resmi genelge, Genelge Coronavirüs Covid 19 %E2%80%93 Yasal Sertifikasyon Hizmetlerinin Ertelenmesinin Uzatılmasına İlişkin Rehberlik 2Güncellendi ile ilgili rehberlik ve düzenleyici kriterler sağlamaktadır.</t>
+          <t>Bu resmi denizcilik sirküleri, Comoros bayraklı gemilerde Tip Onayları ve İdarenin Memnuniyetine İlişkin Kriterler ile ilgili yönergeleri ve idari prosedürleri tanımlamaktadır.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>1. İlgili genelgeyi gemideki sirküler klasörüne ekleyerek zabitlere tebliğ edin. 2. Genelgede belirtilen teknik şartları PSC denetimleri öncesinde kontrol listesine ekleyin.</t>
         </is>
       </c>
     </row>

</xml_diff>